<commit_message>
Finalize local attendance system
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/static/templates/member-import-template.xlsx
+++ b/backend/src/main/resources/static/templates/member-import-template.xlsx
@@ -40,7 +40,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,8 +62,13 @@
         <fgColor rgb="00F3F6FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -85,11 +90,25 @@
         <color rgb="00D9E2EC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -105,6 +124,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -180,31 +205,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Codex</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>必填。系统会按学号判断新增或更新已有成员。</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>必填。成员姓名。</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>可选。格式为 2007级 到 2057级。</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,104 +500,104 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>学号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>姓名</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>手机号</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>专业</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>学院</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>年级</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>QQ</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>202612340001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>张三</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>13800000000</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>计算机科学与技术</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>信息工程学院</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>2026级</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>123456789</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>202612340002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>李四</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>13900000000</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>软件工程</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>信息工程学院</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>2025级</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>987654321</t>
         </is>
@@ -611,7 +611,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>